<commit_message>
Generar Excel plano 2018-2026 para los 11 tramos
- Tabla única: Descripción, Unidad, Fecha, INICIO (KM), FIN (KM), METRADO
- Excel maestro reportes_tramos_2018_2026.xlsx (1 hoja por tramo + resumen)
- Archivo individual tramo_*.xlsx por cada tramo
- FIN en blanco se mantiene vacío tal cual fuente

Co-authored-by: NicolasCutire <NicolasCutire@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/extracted/reports/tramos_filtrado_estricto/tramo_282+280_282+400.xlsx
+++ b/extracted/reports/tramos_filtrado_estricto/tramo_282+280_282+400.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,16 +30,27 @@
       <color rgb="001F4E79"/>
       <sz val="14"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -47,13 +58,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4B4B4"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4B4B4"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4B4B4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4B4B4"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,8 +447,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -432,14 +469,46 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Filtro: FIN completo contenido en tramo; FIN en blanco si INICIO cae en tramo | Total registros: 0</t>
+          <t>Periodo 2018-2026 | Total registros: 0</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Sin registros dentro del tramo evaluado.</t>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>INICIO (KM)</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>FIN (KM)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>METRADO</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sin registros dentro del tramo evaluado (2018-2026).</t>
         </is>
       </c>
     </row>
@@ -447,7 +516,7 @@
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A5:F5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>